<commit_message>
Add replacement URLs for dead DataON pages in Excel results
Added column H '새 URL (대체)' with found replacement URLs for
11 rows where DataON pages returned 404. New URL mapping:
- intro01.do (About/Mission/OAIS/Scope) -> outline.do or mgmtPolicy.do
- intro03.do (History) -> history.do
- intro02.do (Services) -> outline.do
- intro07.do (Cooperated orgs) -> assnOrg.do
- intro08.do (Org chart) -> mgmtPolicy.do
- intro09.do (Metadata schema) -> catalog_summary.do

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DataON_URL_Check_Results.xlsx
+++ b/DataON_URL_Check_Results.xlsx
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -88,6 +93,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -464,6 +472,7 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -502,6 +511,11 @@
           <t>DataON 내 페이지 여부</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>새 URL (대체)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -539,6 +553,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/outline.do</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -650,6 +669,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/history.do</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -687,6 +711,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/outline.do</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -724,6 +753,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/assnOrg.do</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1279,6 +1313,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/outline.do</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1723,6 +1762,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/mgmtPolicy.do</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2130,6 +2174,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/mgmtPolicy.do</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2685,6 +2734,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/mgmtPolicy.do</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2833,6 +2887,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/intro/mgmtPolicy.do</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2870,6 +2929,11 @@
           <t>예 (DataON)</t>
         </is>
       </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/catalog_summary.do</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -3978,6 +4042,11 @@
       <c r="G95" s="3" t="inlineStr">
         <is>
           <t>예 (DataON)</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>https://dataon.kisti.re.kr/catalog_summary.do</t>
         </is>
       </c>
     </row>

</xml_diff>